<commit_message>
Enhance alert data provenance and catalogue UI
</commit_message>
<xml_diff>
--- a/data/source/alerts-ds.xlsx
+++ b/data/source/alerts-ds.xlsx
@@ -981,7 +981,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Tank Temperature Stable</t>
+          <t>Temperature Stable</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Tank Temperature Stable</t>
+          <t>Temperature Stable</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -4981,7 +4981,7 @@
         </is>
       </c>
       <c r="J62" s="5" t="n">
-        <v>45335</v>
+        <v>45672</v>
       </c>
       <c r="K62" s="4" t="inlineStr">
         <is>
@@ -5058,7 +5058,7 @@
         </is>
       </c>
       <c r="J63" s="5" t="n">
-        <v>45336</v>
+        <v>45702</v>
       </c>
       <c r="K63" s="4" t="inlineStr">
         <is>
@@ -5136,7 +5136,7 @@
         </is>
       </c>
       <c r="J64" s="5" t="n">
-        <v>45337</v>
+        <v>45732</v>
       </c>
       <c r="K64" s="4" t="inlineStr">
         <is>
@@ -5217,7 +5217,7 @@
         </is>
       </c>
       <c r="J65" s="5" t="n">
-        <v>45338</v>
+        <v>45762</v>
       </c>
       <c r="K65" s="4" t="inlineStr">
         <is>
@@ -5296,7 +5296,7 @@
         </is>
       </c>
       <c r="J66" s="5" t="n">
-        <v>45339</v>
+        <v>45792</v>
       </c>
       <c r="K66" s="4" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
         </is>
       </c>
       <c r="J67" s="5" t="n">
-        <v>45340</v>
+        <v>45822</v>
       </c>
       <c r="K67" s="4" t="inlineStr">
         <is>
@@ -5452,7 +5452,7 @@
         </is>
       </c>
       <c r="J68" s="5" t="n">
-        <v>45341</v>
+        <v>45852</v>
       </c>
       <c r="K68" s="4" t="inlineStr">
         <is>
@@ -5531,7 +5531,7 @@
         </is>
       </c>
       <c r="J69" s="5" t="n">
-        <v>45342</v>
+        <v>45882</v>
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
@@ -5611,7 +5611,7 @@
         </is>
       </c>
       <c r="J70" s="5" t="n">
-        <v>45343</v>
+        <v>45912</v>
       </c>
       <c r="K70" s="4" t="inlineStr">
         <is>
@@ -5691,7 +5691,7 @@
         </is>
       </c>
       <c r="J71" s="5" t="n">
-        <v>45344</v>
+        <v>45942</v>
       </c>
       <c r="K71" s="4" t="inlineStr">
         <is>
@@ -5769,7 +5769,7 @@
         </is>
       </c>
       <c r="J72" s="5" t="n">
-        <v>45345</v>
+        <v>45972</v>
       </c>
       <c r="K72" s="4" t="inlineStr">
         <is>
@@ -5846,7 +5846,7 @@
         </is>
       </c>
       <c r="J73" s="5" t="n">
-        <v>45346</v>
+        <v>46002</v>
       </c>
       <c r="K73" s="4" t="inlineStr">
         <is>
@@ -5924,7 +5924,7 @@
         </is>
       </c>
       <c r="J74" s="5" t="n">
-        <v>45347</v>
+        <v>46032</v>
       </c>
       <c r="K74" s="4" t="inlineStr">
         <is>
@@ -6005,7 +6005,7 @@
         </is>
       </c>
       <c r="J75" s="5" t="n">
-        <v>45348</v>
+        <v>46062</v>
       </c>
       <c r="K75" s="4" t="inlineStr">
         <is>
@@ -6084,7 +6084,7 @@
         </is>
       </c>
       <c r="J76" s="5" t="n">
-        <v>45349</v>
+        <v>46092</v>
       </c>
       <c r="K76" s="4" t="inlineStr">
         <is>

</xml_diff>